<commit_message>
update manual translation exports 2026-06-26T14:19:36
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,88 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-26T14:19:36</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Untitled</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/38be8c8a654d801fad96c5603f7f69f5</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-801f-ad96-c5603f7f69f5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-26T14:19:36</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Untitled</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/38be8c8a654d80c1a227fbff84e12200</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-80c1-a227-fbff84e12200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update literature workflow 2026-06-26T14:27:14
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,40 +474,70 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>use_type</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>related_chapter</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>reading_status</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>translation_status</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>derived_translation_status</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>processing_status</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>translation_status</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>use_type</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>related_chapter</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>derived_processing_status</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>claim_supported</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>notion_writeback_status</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>material_pack_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
         </is>
@@ -516,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T14:19:36</t>
+          <t>2026-06-26T14:27:14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -535,20 +565,42 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>待翻译</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr">
         <is>
+          <t>待补充信息</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>待补充信息</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr">
+        <is>
           <t>https://app.notion.com/p/38be8c8a654d801fad96c5603f7f69f5</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>38be8c8a-654d-801f-ad96-c5603f7f69f5</t>
         </is>
@@ -557,7 +609,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T14:19:36</t>
+          <t>2026-06-26T14:27:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -576,20 +628,42 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>待翻译</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
+          <t>待补充信息</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>待补充信息</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
+        <is>
           <t>https://app.notion.com/p/38be8c8a654d80c1a227fbff84e12200</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>38be8c8a-654d-80c1-a227-fbff84e12200</t>
         </is>

</xml_diff>

<commit_message>
update literature workflow 2026-06-26T14:31:35
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -546,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T14:27:14</t>
+          <t>2026-06-26T14:31:35</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -591,7 +591,7 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -609,7 +609,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T14:27:14</t>
+          <t>2026-06-26T14:31:35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -654,7 +654,7 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>

</xml_diff>

<commit_message>
update literature workflow 2026-06-26T14:32:16
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -546,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T14:31:35</t>
+          <t>2026-06-26T14:32:16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -609,7 +609,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T14:31:35</t>
+          <t>2026-06-26T14:32:16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T17:46:06
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:Z7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,562 @@
       <c r="Z1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:46:06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The link between perceived human resource management practices, engagement and employee behaviour: a moderated mediation model</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>K. Alfes; A. D. Shantz; C. Truss; E. C. Soane</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>10.1080/09585192.2012.679950</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>This study contributes to our understanding of the mediating and moderating processes through which human resource management practices are linked with behavioural outcomes. We developed and tested a moderated mediation model linking perceived human resource management practices to organisational citizenship behaviour and turnover intentions. Drawing on social exchange theory, our model posits that the effect of perceived human resource management practices on both outcome variables is mediated by levels of employee engagement, while the relationship between employee engagement and both outcome variables is moderated by perceived organisational support and leader-member exchange. Overall, data from 297 employees in a service sector organisation in the UK support this model. This suggests that the enactment of positive behavioural outcomes, as a consequence of engagement, largely depends on the wider organisational climate and employees’ relationship with their line manager. Implications for practice and directions for future research are discussed.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/The-link-between-perceived-human-resource-management-practices-engagement-and-employee-behaviour-a-38be8c8a654d8156b64feb22e71f3dc6</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-8156-b64f-eb22e71f3dc6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:46:06</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Allocative efficiency in public research funding: Can bibliometrics help?</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Giovanni Abramo; Ciriaco Andrea D’Angelo; Alessandro Caprasecca</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>10.1016/j.respol.2008.11.001</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>The use of outcome control modes of research evaluation exercises is ever more frequent. They are conceived as tools to stimulate increased levels of research productivity, and to guide choices in allocating components of government research budgets for publicly funded institutions. There are several contributions in the literature that compare the different methodological approaches that policy makers could adopt for these exercises, however the comparisons are limited to only a few disciplines. This work, examining the case of the whole of the “hard sciences” of the Italian academic system, makes a comparison between results obtained from peer review type of evaluations (as adopted by the Ministry of Universities and Research) and those possible from a bibliometric approach (as developed by the authors). The aim is to understand to what extent bibliometric methodology, which is noted as relatively inexpensive, time-saving and exhaustive, can complement and integrate peer review methodology in research evaluation.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>To Read</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Allocative-efficiency-in-public-research-funding-Can-bibliometrics-help-38be8c8a654d81818002f18f597e778a</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-8181-8002-f18f597e778a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:46:06</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Consumer attitudes toward marketplace globalization: Structure, antecedents and consequences</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Dana L. Alden; Jan-Benedict E.M. Steenkamp; Rajeev Batra</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>10.1016/j.ijresmar.2006.01.010</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>This study examines relationships between a new measure of consumer attitudes toward consumption alternatives resulting from market globalization, several attitudinal antecedents (materialism, susceptibility to normative influence and consumer ethnocentrism), and a hypothesized consequence of these attitudes — preference for global brands. Following validation of the new measure in three culturally distinct markets, South Korea, the US, and China, the hypothesized antecedents and consequence are tested in South Korea. Empirical findings broadly support hypotheses and provide important implications for future research on market globalization.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>To Read</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Consumer-attitudes-toward-marketplace-globalization-Structure-antecedents-and-consequences-38be8c8a654d8127b61bfa21295ef56e</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-8127-b61b-fa21295ef56e</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:46:06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The Brand Relationship Spectrum: The Key to the Brand Architecture Challenge</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>David A. Aaker; Erich Joachimsthaler</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>10.1177/000812560004200401</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/The-Brand-Relationship-Spectrum-The-Key-to-the-Brand-Architecture-Challenge-38be8c8a654d81f69706d64fa491b0b7</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-81f6-9706-d64fa491b0b7</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:46:06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Measuring Brand Equity Across Products and Markets</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>David A. Aaker</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>10.2307/41165845</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Measuring-Brand-Equity-Across-Products-and-Markets-38be8c8a654d81f0b640c6749576402a</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-81f0-b640-c6749576402a</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:46:06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Leveraging the Corporate Brand</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>David A Aaker</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>待翻译</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Leveraging-the-Corporate-Brand-38be8c8a654d81b586f5ff72a1a20d98</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>38be8c8a-654d-81b5-86f5-ff72a1a20d98</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T17:53:16
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T17:46:06</t>
+          <t>2026-06-26T17:53:16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>to-notion</t>
+          <t>to-notion, Method, Theory, Survey</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T17:46:06</t>
+          <t>2026-06-26T17:53:16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -685,7 +685,7 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>to-notion</t>
+          <t>to-notion, Method, Experiment</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -743,7 +743,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T17:46:06</t>
+          <t>2026-06-26T17:53:16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -781,7 +781,7 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>to-notion</t>
+          <t>to-notion, Survey</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -839,7 +839,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T17:46:06</t>
+          <t>2026-06-26T17:53:16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -931,7 +931,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T17:46:06</t>
+          <t>2026-06-26T17:53:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T17:46:06</t>
+          <t>2026-06-26T17:53:16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T18:11:55
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T17:58:40</t>
+          <t>2026-06-26T18:11:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -575,7 +575,11 @@
           <t>2013</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>The International Journal of Human Resource Management</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>10.1080/09585192.2012.679950</t>
@@ -589,18 +593,14 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>to-notion, Method, Theory, Survey</t>
+          <t>to-notion</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>待翻译</t>
@@ -635,19 +635,19 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>https://app.notion.com/p/The-link-between-perceived-human-resource-management-practices-engagement-and-employee-behaviour-a-38be8c8a654d8156b64feb22e71f3dc6</t>
+          <t>https://app.notion.com/p/The-link-between-perceived-human-resource-management-practices-engagement-and-employee-behaviour-a-38be8c8a654d815c8b72cca5fd0666fb</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>38be8c8a-654d-8156-b64f-eb22e71f3dc6</t>
+          <t>38be8c8a-654d-815c-8b72-cca5fd0666fb</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T17:58:40</t>
+          <t>2026-06-26T18:11:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -671,7 +671,11 @@
           <t>2009</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Research Policy</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>10.1016/j.respol.2008.11.001</t>
@@ -685,18 +689,14 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>to-notion, Method, Experiment</t>
+          <t>to-notion</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>To Read</t>
-        </is>
-      </c>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>待翻译</t>
@@ -731,19 +731,19 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>https://app.notion.com/p/Allocative-efficiency-in-public-research-funding-Can-bibliometrics-help-38be8c8a654d81818002f18f597e778a</t>
+          <t>https://app.notion.com/p/Allocative-efficiency-in-public-research-funding-Can-bibliometrics-help-38be8c8a654d81ee87ecf054b8ee4a43</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>38be8c8a-654d-8181-8002-f18f597e778a</t>
+          <t>38be8c8a-654d-81ee-87ec-f054b8ee4a43</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T17:58:40</t>
+          <t>2026-06-26T18:11:55</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -767,7 +767,11 @@
           <t>2006</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>International Journal of Research in Marketing</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>10.1016/j.ijresmar.2006.01.010</t>
@@ -781,18 +785,14 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>to-notion, Survey</t>
+          <t>to-notion</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>To Read</t>
-        </is>
-      </c>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>待翻译</t>
@@ -827,19 +827,19 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>https://app.notion.com/p/Consumer-attitudes-toward-marketplace-globalization-Structure-antecedents-and-consequences-38be8c8a654d8127b61bfa21295ef56e</t>
+          <t>https://app.notion.com/p/Consumer-attitudes-toward-marketplace-globalization-Structure-antecedents-and-consequences-38be8c8a654d8181b104dba51bded1a6</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>38be8c8a-654d-8127-b61b-fa21295ef56e</t>
+          <t>38be8c8a-654d-8181-b104-dba51bded1a6</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T17:58:40</t>
+          <t>2026-06-26T18:11:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -863,7 +863,11 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>California Management Review</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>10.1177/000812560004200401</t>
@@ -880,11 +884,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
           <t>待翻译</t>
@@ -919,19 +919,19 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>https://app.notion.com/p/The-Brand-Relationship-Spectrum-The-Key-to-the-Brand-Architecture-Challenge-38be8c8a654d81f69706d64fa491b0b7</t>
+          <t>https://app.notion.com/p/The-Brand-Relationship-Spectrum-The-Key-to-the-Brand-Architecture-Challenge-38be8c8a654d81bc87b3c0d49f35522c</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>38be8c8a-654d-81f6-9706-d64fa491b0b7</t>
+          <t>38be8c8a-654d-81bc-87b3-c0d49f35522c</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T17:58:40</t>
+          <t>2026-06-26T18:11:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -955,7 +955,11 @@
           <t>1996</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>California Management Review</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>10.2307/41165845</t>
@@ -972,11 +976,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>待翻译</t>
@@ -1011,19 +1011,19 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>https://app.notion.com/p/Measuring-Brand-Equity-Across-Products-and-Markets-38be8c8a654d81f0b640c6749576402a</t>
+          <t>https://app.notion.com/p/Measuring-Brand-Equity-Across-Products-and-Markets-38be8c8a654d81a2b11cf39eb2afaab8</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>38be8c8a-654d-81f0-b640-c6749576402a</t>
+          <t>38be8c8a-654d-81a2-b11c-f39eb2afaab8</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T17:58:40</t>
+          <t>2026-06-26T18:11:55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1056,11 +1056,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
           <t>待翻译</t>
@@ -1095,12 +1091,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>https://app.notion.com/p/Leveraging-the-Corporate-Brand-38be8c8a654d81b586f5ff72a1a20d98</t>
+          <t>https://app.notion.com/p/Leveraging-the-Corporate-Brand-38be8c8a654d815fbed4f3c2c82d9e0b</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>38be8c8a-654d-81b5-86f5-ff72a1a20d98</t>
+          <t>38be8c8a-654d-815f-bed4-f3c2c82d9e0b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T18:16:21
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:11:55</t>
+          <t>2026-06-26T18:16:21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:11:55</t>
+          <t>2026-06-26T18:16:21</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -743,7 +743,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:11:55</t>
+          <t>2026-06-26T18:16:21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -839,7 +839,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:11:55</t>
+          <t>2026-06-26T18:16:21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -931,7 +931,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:11:55</t>
+          <t>2026-06-26T18:16:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:11:55</t>
+          <t>2026-06-26T18:16:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1078,7 +1078,11 @@
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>53535353</t>
+        </is>
+      </c>
       <c r="W7" t="inlineStr">
         <is>
           <t>skipped_existing_or_no_fields</t>

</xml_diff>

<commit_message>
update content-aware literature exports
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:AI7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,20 +529,65 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
+          <t>evaluation</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>block_count</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>comment_count</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>page_body_preview</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>has_page_body</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>has_comments</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>in_all_material_pack</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>in_literature_review_pack</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>in_theory_pack</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
           <t>notion_writeback_status</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>material_pack_status</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
         </is>
@@ -551,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:16:21</t>
+          <t>2026-06-26T18:24:06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -623,22 +668,45 @@
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr">
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="inlineStr">
         <is>
           <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>generated</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>https://app.notion.com/p/The-link-between-perceived-human-resource-management-practices-engagement-and-employee-behaviour-a-38be8c8a654d815c8b72cca5fd0666fb</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>38be8c8a-654d-815c-8b72-cca5fd0666fb</t>
         </is>
@@ -647,7 +715,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:16:21</t>
+          <t>2026-06-26T18:24:06</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -719,22 +787,45 @@
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="inlineStr">
         <is>
           <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>generated</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
         <is>
           <t>https://app.notion.com/p/Allocative-efficiency-in-public-research-funding-Can-bibliometrics-help-38be8c8a654d81ee87ecf054b8ee4a43</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>38be8c8a-654d-81ee-87ec-f054b8ee4a43</t>
         </is>
@@ -743,7 +834,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:16:21</t>
+          <t>2026-06-26T18:24:06</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -815,22 +906,45 @@
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="inlineStr">
         <is>
           <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>generated</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>https://app.notion.com/p/Consumer-attitudes-toward-marketplace-globalization-Structure-antecedents-and-consequences-38be8c8a654d8181b104dba51bded1a6</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>38be8c8a-654d-8181-b104-dba51bded1a6</t>
         </is>
@@ -839,7 +953,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:16:21</t>
+          <t>2026-06-26T18:24:06</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -907,22 +1021,45 @@
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr">
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="inlineStr">
         <is>
           <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="AG5" t="inlineStr">
         <is>
           <t>generated</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>https://app.notion.com/p/The-Brand-Relationship-Spectrum-The-Key-to-the-Brand-Architecture-Challenge-38be8c8a654d81bc87b3c0d49f35522c</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AI5" t="inlineStr">
         <is>
           <t>38be8c8a-654d-81bc-87b3-c0d49f35522c</t>
         </is>
@@ -931,7 +1068,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:16:21</t>
+          <t>2026-06-26T18:24:06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -999,22 +1136,45 @@
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="inlineStr">
         <is>
           <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
         <is>
           <t>generated</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>https://app.notion.com/p/Measuring-Brand-Equity-Across-Products-and-Markets-38be8c8a654d81a2b11cf39eb2afaab8</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>38be8c8a-654d-81a2-b11c-f39eb2afaab8</t>
         </is>
@@ -1023,7 +1183,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:16:21</t>
+          <t>2026-06-26T18:24:06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1085,20 +1245,51 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
+          <t>98765</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>你好再见</t>
+        </is>
+      </c>
+      <c r="AA7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
           <t>skipped_existing_or_no_fields</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="AG7" t="inlineStr">
         <is>
           <t>generated</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AH7" t="inlineStr">
         <is>
           <t>https://app.notion.com/p/Leveraging-the-Corporate-Brand-38be8c8a654d815fbed4f3c2c82d9e0b</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>38be8c8a-654d-815f-bed4-f3c2c82d9e0b</t>
         </is>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T18:41:29
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:33:25</t>
+          <t>2026-06-26T18:41:29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -715,7 +715,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:33:25</t>
+          <t>2026-06-26T18:41:29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -834,7 +834,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:33:25</t>
+          <t>2026-06-26T18:41:29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -953,7 +953,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:33:25</t>
+          <t>2026-06-26T18:41:29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -995,8 +995,16 @@
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>概念定义</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>研究方法</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
@@ -1068,7 +1076,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:33:25</t>
+          <t>2026-06-26T18:41:29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1110,8 +1118,16 @@
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>机制解释</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>理论基础</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
@@ -1157,7 +1173,7 @@
         <v>0</v>
       </c>
       <c r="AE6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
@@ -1183,7 +1199,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:33:25</t>
+          <t>2026-06-26T18:41:29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1213,8 +1229,16 @@
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>概念定义</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>文献综述</t>
+        </is>
+      </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
@@ -1269,7 +1293,7 @@
         <v>1</v>
       </c>
       <c r="AD7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE7" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T18:50:39
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:41:29</t>
+          <t>2026-06-26T18:50:39</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -715,7 +715,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:41:29</t>
+          <t>2026-06-26T18:50:39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -834,7 +834,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:41:29</t>
+          <t>2026-06-26T18:50:39</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -953,7 +953,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:41:29</t>
+          <t>2026-06-26T18:50:39</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1076,7 +1076,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:41:29</t>
+          <t>2026-06-26T18:50:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:41:29</t>
+          <t>2026-06-26T18:50:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1273,14 +1273,15 @@
         </is>
       </c>
       <c r="X7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y7" t="n">
         <v>1</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>你好再见</t>
+          <t>你好再见
+as i was a child ,i would like to become a superstar.therefore, i only get a doll from my parents.</t>
         </is>
       </c>
       <c r="AA7" t="b">

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T19:01:35
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:58:21</t>
+          <t>2026-06-26T19:01:35</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -723,7 +723,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:58:21</t>
+          <t>2026-06-26T19:01:35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -850,7 +850,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:58:21</t>
+          <t>2026-06-26T19:01:35</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:58:21</t>
+          <t>2026-06-26T19:01:35</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:58:21</t>
+          <t>2026-06-26T19:01:35</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1231,7 +1231,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:58:21</t>
+          <t>2026-06-26T19:01:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>